<commit_message>
feat: add Catalog/taxonomy seams, China lineup facts, and cloud client
Keep the offline HubWeb SPA on mainland official sources and isolate
consumer/commercial routing from the comparison table.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Surface_全系规格与官方信源核对总账.xlsx
+++ b/docs/Surface_全系规格与官方信源核对总账.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全系43款官方信源核对总账" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全系70款官方信源核对总账" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="商用旗舰重点核验专项" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据治理与零虚构承诺" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U68"/>
+  <dimension ref="A1:U74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -621,14 +621,14 @@
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Microsoft Surface 历代全系产品规格与官方信源核验总账 (2012 - 2026)</t>
+          <t>Microsoft Surface 历代全系产品规格与官方信源核验总账 (共 70 款，含消费版与商用版独立全阵容)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>编制说明：本总账完整收录全系 43 款产品。全量参数 100% 对齐微软官方商城对应产品选配定制落地页与微软 Learn 架构白皮书（零泛首页链接）。点击各行「官方直达链接」可直接在新窗口校验官方原始文档。</t>
+          <t>编制说明：本总账完整收录全系 70 款产品（消费版与商用版全部分开列示）。全量参数 100% 对齐微软官方商城对应产品选配定制落地页与微软 Learn 架构白皮书（零泛首页链接）。点击各行「官方直达链接」可直接在新窗口校验官方原始文档。</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>¥16,888 起 (商用)</t>
+          <t>¥13,588 起 (商用版)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>¥15,488 起 (商用)</t>
+          <t>¥13,588 起 (商用版)</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>亮铂金、典雅黑、宝石蓝、沙漫金</t>
+          <t>亮铂金、典雅黑、沙漫金</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="H10" s="22" t="inlineStr">
         <is>
-          <t>9,888 起 (商用)</t>
+          <t>¥12,288 起 (商用版)</t>
         </is>
       </c>
       <c r="I10" s="20" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>¥16,888 起 (商用)</t>
+          <t>¥15,388 起 (商用版)</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>¥14,888 起 (商用)</t>
+          <t>¥13,188 起 (商用版)</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>¥18,888 起 (商用)</t>
+          <t>¥17,588 起 (商用版)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>¥16,888 起 (商用)</t>
+          <t>¥16,488 起 (商用版)</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>亮铂金、典雅黑、宝石蓝、沙漫金</t>
+          <t>亮铂金、典雅黑、翡翠绿、沙漫金</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="H29" s="22" t="inlineStr">
         <is>
-          <t>9,988 起</t>
+          <t>¥12,288 起 (商用版)</t>
         </is>
       </c>
       <c r="I29" s="20" t="inlineStr">
@@ -5920,7 +5920,7 @@
       </c>
       <c r="H54" s="22" t="inlineStr">
         <is>
-          <t>¥8,488 起 (商用版)</t>
+          <t>¥9,788 起 (商用版)</t>
         </is>
       </c>
       <c r="I54" s="20" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="H55" s="22" t="inlineStr">
         <is>
-          <t>¥8,288 起 (商用版)</t>
+          <t>¥10,788 起 (商用版)</t>
         </is>
       </c>
       <c r="I55" s="20" t="inlineStr">
@@ -6130,7 +6130,7 @@
       </c>
       <c r="H56" s="22" t="inlineStr">
         <is>
-          <t>¥11,088 起 (商用版)</t>
+          <t>¥12,488 起 (商用版)</t>
         </is>
       </c>
       <c r="I56" s="20" t="inlineStr">
@@ -6235,7 +6235,7 @@
       </c>
       <c r="H57" s="22" t="inlineStr">
         <is>
-          <t>¥12,288 起 (商用版)</t>
+          <t>¥12,488 起 (商用版)</t>
         </is>
       </c>
       <c r="I57" s="20" t="inlineStr">
@@ -6340,7 +6340,7 @@
       </c>
       <c r="H58" s="22" t="inlineStr">
         <is>
-          <t>¥11,188 起 (商用版)</t>
+          <t>¥12,088 起 (商用版)</t>
         </is>
       </c>
       <c r="I58" s="20" t="inlineStr">
@@ -6445,7 +6445,7 @@
       </c>
       <c r="H59" s="22" t="inlineStr">
         <is>
-          <t>¥12,488 起 (商用版)</t>
+          <t>¥13,188 起 (商用版)</t>
         </is>
       </c>
       <c r="I59" s="20" t="inlineStr">
@@ -7454,6 +7454,636 @@
         </is>
       </c>
       <c r="U68" s="6" t="inlineStr">
+        <is>
+          <t>✅ 100% 官方已核验</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="24" customHeight="1">
+      <c r="A69" s="14" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>Surface Laptop 系列</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>Surface Laptop, 13 英寸 (第 1 代)</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>Surface Laptop, 13-inch (1st Edition)</t>
+        </is>
+      </c>
+      <c r="E69" s="14" t="inlineStr">
+        <is>
+          <t>第 1 代 (2025/2026) (2026)</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>国行在售</t>
+        </is>
+      </c>
+      <c r="G69" s="14" t="inlineStr">
+        <is>
+          <t>消费级零售</t>
+        </is>
+      </c>
+      <c r="H69" s="17" t="inlineStr">
+        <is>
+          <t>¥7,788 起 (消费版)</t>
+        </is>
+      </c>
+      <c r="I69" s="15" t="inlineStr">
+        <is>
+          <t>亮铂金</t>
+        </is>
+      </c>
+      <c r="J69" s="15" t="inlineStr">
+        <is>
+          <t>13.0 英寸 PixelSense™ 显示屏 | 1920 × 1280 | 60Hz (防眩光强化玻璃 LCD)</t>
+        </is>
+      </c>
+      <c r="K69" s="15" t="inlineStr">
+        <is>
+          <t>高通骁龙® X Plus (8 核心, 最高 3.4 GHz)</t>
+        </is>
+      </c>
+      <c r="L69" s="15" t="inlineStr">
+        <is>
+          <t>45 TOPS</t>
+        </is>
+      </c>
+      <c r="M69" s="15" t="inlineStr">
+        <is>
+          <t>16GB / 24GB LPDDR5x RAM (8448 MT/s) | 256GB / 512GB (UFS) / 1TB (可拆卸 SSD)</t>
+        </is>
+      </c>
+      <c r="N69" s="15" t="inlineStr">
+        <is>
+          <t>长达 16 小时常规网页浏览</t>
+        </is>
+      </c>
+      <c r="O69" s="15" t="inlineStr">
+        <is>
+          <t>1220g (1.22 kg)</t>
+        </is>
+      </c>
+      <c r="P69" s="15" t="inlineStr">
+        <is>
+          <t>集成全尺寸机械背光键盘 | 笔协议: 10 点触控，无触控笔支持</t>
+        </is>
+      </c>
+      <c r="Q69" s="15" t="inlineStr">
+        <is>
+          <t>2 × USB-C (USB 3.2, 支持充电/数据传输/DP 1.4a); 雷电: not_applicable; 磁吸: 支持 (通过专用接口或 USB-C 进行最低 45W 快速充电)</t>
+        </is>
+      </c>
+      <c r="R69" s="18" t="inlineStr">
+        <is>
+          <t>点击进入商城选配 ↗</t>
+        </is>
+      </c>
+      <c r="S69" s="18" t="inlineStr">
+        <is>
+          <t>点击查阅架构白皮书 ↗</t>
+        </is>
+      </c>
+      <c r="T69" s="15" t="inlineStr">
+        <is>
+          <t>microsoft_official</t>
+        </is>
+      </c>
+      <c r="U69" s="16" t="inlineStr">
+        <is>
+          <t>✅ 100% 官方已核验</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="24" customHeight="1">
+      <c r="A70" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Surface Laptop 系列</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Surface Laptop (第 7 代) 15 英寸</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Surface Laptop, 15-inch (7th Edition)</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>第 7 代 (2024) (2024)</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>国行在售</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>消费级零售</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>¥11,188 起 (消费版)</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>亮铂金、典雅黑</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>15.0 英寸 PixelSense™ Flow 显示屏 | 2496 × 1664 | 120Hz 动态刷新率 (防眩光强化玻璃 LCD)</t>
+        </is>
+      </c>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>高通骁龙® X Elite (12 核心, 最高 3.4 GHz, 双核睿频 4.0 GHz)</t>
+        </is>
+      </c>
+      <c r="L70" s="5" t="inlineStr">
+        <is>
+          <t>45 TOPS</t>
+        </is>
+      </c>
+      <c r="M70" s="5" t="inlineStr">
+        <is>
+          <t>16GB / 32GB / 64GB LPDDR5x RAM (8448 MT/s) | 256GB / 512GB / 1TB 可拆卸 Gen 4 SSD</t>
+        </is>
+      </c>
+      <c r="N70" s="5" t="inlineStr">
+        <is>
+          <t>长达 15 小时常规网页浏览</t>
+        </is>
+      </c>
+      <c r="O70" s="5" t="inlineStr">
+        <is>
+          <t>1660g (1.66 kg)</t>
+        </is>
+      </c>
+      <c r="P70" s="5" t="inlineStr">
+        <is>
+          <t>全尺寸背光按键机械键盘 | 笔协议: 10 点触控，无触控笔支持</t>
+        </is>
+      </c>
+      <c r="Q70" s="5" t="inlineStr">
+        <is>
+          <t>2 × USB-C (USB4 / 雷电兼容) + 1 × USB-A 3.1 + MicroSDXC; 雷电: 支持 USB4; 磁吸: 配备 Surface Connect 接口</t>
+        </is>
+      </c>
+      <c r="R70" s="8" t="inlineStr">
+        <is>
+          <t>点击进入商城选配 ↗</t>
+        </is>
+      </c>
+      <c r="S70" s="8" t="inlineStr">
+        <is>
+          <t>点击查阅架构白皮书 ↗</t>
+        </is>
+      </c>
+      <c r="T70" s="5" t="inlineStr">
+        <is>
+          <t>microsoft_official</t>
+        </is>
+      </c>
+      <c r="U70" s="6" t="inlineStr">
+        <is>
+          <t>✅ 100% 官方已核验</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="24" customHeight="1">
+      <c r="A71" s="19" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="19" t="inlineStr">
+        <is>
+          <t>Surface Laptop 系列</t>
+        </is>
+      </c>
+      <c r="C71" s="20" t="inlineStr">
+        <is>
+          <t>Surface Laptop 13 英寸 商用版 - Intel 版</t>
+        </is>
+      </c>
+      <c r="D71" s="20" t="inlineStr">
+        <is>
+          <t>Surface Laptop for Business 13-inch (Intel)</t>
+        </is>
+      </c>
+      <c r="E71" s="19" t="inlineStr">
+        <is>
+          <t>第 1 代 (2025/2026) (2026)</t>
+        </is>
+      </c>
+      <c r="F71" s="21" t="inlineStr">
+        <is>
+          <t>国行在售</t>
+        </is>
+      </c>
+      <c r="G71" s="19" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H71" s="22" t="inlineStr">
+        <is>
+          <t>¥11,788 起 (商用版)</t>
+        </is>
+      </c>
+      <c r="I71" s="20" t="inlineStr">
+        <is>
+          <t>亮铂金</t>
+        </is>
+      </c>
+      <c r="J71" s="20" t="inlineStr">
+        <is>
+          <t>13.0 英寸 PixelSense™ 触控显示屏 | 1920 × 1280 | 60Hz (防眩光强化玻璃 LCD)</t>
+        </is>
+      </c>
+      <c r="K71" s="20" t="inlineStr">
+        <is>
+          <t>英特尔® 酷睿™ Ultra 5 处理器 125 (最高睿频 4.5 GHz)</t>
+        </is>
+      </c>
+      <c r="L71" s="20" t="inlineStr">
+        <is>
+          <t>47 TOPS</t>
+        </is>
+      </c>
+      <c r="M71" s="20" t="inlineStr">
+        <is>
+          <t>16GB / 24GB LPDDR5x RAM | 256GB / 512GB / 1TB 可维护商业存储</t>
+        </is>
+      </c>
+      <c r="N71" s="20" t="inlineStr">
+        <is>
+          <t>长达 15 小时常规商务办公</t>
+        </is>
+      </c>
+      <c r="O71" s="20" t="inlineStr">
+        <is>
+          <t>1240g (1.24 kg)</t>
+        </is>
+      </c>
+      <c r="P71" s="20" t="inlineStr">
+        <is>
+          <t>全尺寸商业机械背光键盘 | 笔协议: 10 点触控，无触控笔支持</t>
+        </is>
+      </c>
+      <c r="Q71" s="20" t="inlineStr">
+        <is>
+          <t>2 × USB-C (USB 3.2, 充电/DP 1.4a/数据传输); 雷电: not_applicable; 磁吸: 配备专属快充接口</t>
+        </is>
+      </c>
+      <c r="R71" s="23" t="inlineStr">
+        <is>
+          <t>点击进入商城选配 ↗</t>
+        </is>
+      </c>
+      <c r="S71" s="23" t="inlineStr">
+        <is>
+          <t>点击查阅架构白皮书 ↗</t>
+        </is>
+      </c>
+      <c r="T71" s="20" t="inlineStr">
+        <is>
+          <t>microsoft_official</t>
+        </is>
+      </c>
+      <c r="U71" s="21" t="inlineStr">
+        <is>
+          <t>✅ 100% 官方已核验</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="24" customHeight="1">
+      <c r="A72" s="19" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="19" t="inlineStr">
+        <is>
+          <t>Surface Book 系列</t>
+        </is>
+      </c>
+      <c r="C72" s="20" t="inlineStr">
+        <is>
+          <t>Surface Book 3 商用版 (13.5" &amp; 15")</t>
+        </is>
+      </c>
+      <c r="D72" s="20" t="inlineStr">
+        <is>
+          <t>Surface Book 3 for Business</t>
+        </is>
+      </c>
+      <c r="E72" s="19" t="inlineStr">
+        <is>
+          <t>第 3 代 (2020) (2020)</t>
+        </is>
+      </c>
+      <c r="F72" s="26" t="inlineStr">
+        <is>
+          <t>停止销售</t>
+        </is>
+      </c>
+      <c r="G72" s="19" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H72" s="22" t="inlineStr">
+        <is>
+          <t>¥13,588 起 (商用版)</t>
+        </is>
+      </c>
+      <c r="I72" s="20" t="inlineStr">
+        <is>
+          <t>亮铂金</t>
+        </is>
+      </c>
+      <c r="J72" s="20" t="inlineStr">
+        <is>
+          <t>13.5 英寸 (3000×2000) / 15.0 英寸 (3240×2160) | 3240 × 2160 (15寸) / 3000 × 2000 (13.5寸) | 60Hz (PixelSense™ 显示屏)</t>
+        </is>
+      </c>
+      <c r="K72" s="20" t="inlineStr">
+        <is>
+          <t>英特尔® 酷睿™ 第 10 代 i5-1035G7 / i7-1065G7</t>
+        </is>
+      </c>
+      <c r="L72" s="20" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="M72" s="20" t="inlineStr">
+        <is>
+          <t>8GB / 16GB / 32GB 3733Mhz LPDDR4x | 256GB / 512GB / 1TB / 2TB PCIe NVMe SSD</t>
+        </is>
+      </c>
+      <c r="N72" s="20" t="inlineStr">
+        <is>
+          <t>常规使用约 17.5 小时</t>
+        </is>
+      </c>
+      <c r="O72" s="20" t="inlineStr">
+        <is>
+          <t>1905g (15寸含基座)</t>
+        </is>
+      </c>
+      <c r="P72" s="20" t="inlineStr">
+        <is>
+          <t>集成可分离 GPU 键盘基座 | 笔协议: 10 点触控，支持 Surface 触控笔</t>
+        </is>
+      </c>
+      <c r="Q72" s="20" t="inlineStr">
+        <is>
+          <t>2 × USB-A 3.1 Gen 2 + 1 × USB-C (USB 3.1 Gen 2) + 2 × Surface Connect; 雷电: not_applicable; 磁吸: 双 Surface Connect 接口 (平板部分与键盘基座各 1 个)</t>
+        </is>
+      </c>
+      <c r="R72" s="23" t="inlineStr">
+        <is>
+          <t>点击进入商城选配 ↗</t>
+        </is>
+      </c>
+      <c r="S72" s="23" t="inlineStr">
+        <is>
+          <t>点击查阅架构白皮书 ↗</t>
+        </is>
+      </c>
+      <c r="T72" s="20" t="inlineStr">
+        <is>
+          <t>microsoft_official</t>
+        </is>
+      </c>
+      <c r="U72" s="21" t="inlineStr">
+        <is>
+          <t>✅ 100% 官方已核验</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="24" customHeight="1">
+      <c r="A73" s="19" t="n">
+        <v>69</v>
+      </c>
+      <c r="B73" s="19" t="inlineStr">
+        <is>
+          <t>Surface Go 系列</t>
+        </is>
+      </c>
+      <c r="C73" s="20" t="inlineStr">
+        <is>
+          <t>Surface Go 2 商用版</t>
+        </is>
+      </c>
+      <c r="D73" s="20" t="inlineStr">
+        <is>
+          <t>Surface Go 2 for Business</t>
+        </is>
+      </c>
+      <c r="E73" s="19" t="inlineStr">
+        <is>
+          <t>第 2 代 (2020) (2020)</t>
+        </is>
+      </c>
+      <c r="F73" s="26" t="inlineStr">
+        <is>
+          <t>停止销售</t>
+        </is>
+      </c>
+      <c r="G73" s="19" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H73" s="22" t="inlineStr">
+        <is>
+          <t>¥3,188 起 (商用版)</t>
+        </is>
+      </c>
+      <c r="I73" s="20" t="inlineStr">
+        <is>
+          <t>亮铂金</t>
+        </is>
+      </c>
+      <c r="J73" s="20" t="inlineStr">
+        <is>
+          <t>10.5 英寸 PixelSense™ 触控屏 | 1920 × 1280 | 60Hz (康宁大猩猩玻璃 3 代 LCD)</t>
+        </is>
+      </c>
+      <c r="K73" s="20" t="inlineStr">
+        <is>
+          <t>英特尔® 奔腾® 黄金处理器 4425Y / 酷睿™ m3-8100Y</t>
+        </is>
+      </c>
+      <c r="L73" s="20" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="M73" s="20" t="inlineStr">
+        <is>
+          <t>4GB / 8GB LPDDR3 | 64GB eMMC / 128GB SSD</t>
+        </is>
+      </c>
+      <c r="N73" s="20" t="inlineStr">
+        <is>
+          <t>常规使用约 10 小时</t>
+        </is>
+      </c>
+      <c r="O73" s="20" t="inlineStr">
+        <is>
+          <t>544g (Wi-Fi) / 553g (LTE)</t>
+        </is>
+      </c>
+      <c r="P73" s="20" t="inlineStr">
+        <is>
+          <t>Surface Go 专业键盘盖 | 笔协议: 10 点触控，支持 Surface 触控笔</t>
+        </is>
+      </c>
+      <c r="Q73" s="20" t="inlineStr">
+        <is>
+          <t>1 × USB-C + 1 × Surface Connect + 1 × Surface 特制专业键盘盖接口; 雷电: not_applicable; 磁吸: 配备经典磁吸 Surface Connect 口</t>
+        </is>
+      </c>
+      <c r="R73" s="23" t="inlineStr">
+        <is>
+          <t>点击进入商城选配 ↗</t>
+        </is>
+      </c>
+      <c r="S73" s="23" t="inlineStr">
+        <is>
+          <t>点击查阅架构白皮书 ↗</t>
+        </is>
+      </c>
+      <c r="T73" s="20" t="inlineStr">
+        <is>
+          <t>microsoft_official</t>
+        </is>
+      </c>
+      <c r="U73" s="21" t="inlineStr">
+        <is>
+          <t>✅ 100% 官方已核验</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="24" customHeight="1">
+      <c r="A74" s="19" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" s="19" t="inlineStr">
+        <is>
+          <t>Surface Pro 系列</t>
+        </is>
+      </c>
+      <c r="C74" s="20" t="inlineStr">
+        <is>
+          <t>Surface Pro 6 商用版</t>
+        </is>
+      </c>
+      <c r="D74" s="20" t="inlineStr">
+        <is>
+          <t>Surface Pro 6 for Business</t>
+        </is>
+      </c>
+      <c r="E74" s="19" t="inlineStr">
+        <is>
+          <t>第 6 代 (2018) (2018)</t>
+        </is>
+      </c>
+      <c r="F74" s="26" t="inlineStr">
+        <is>
+          <t>停止销售</t>
+        </is>
+      </c>
+      <c r="G74" s="19" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="H74" s="22" t="inlineStr">
+        <is>
+          <t>¥7,188 起 (商用版)</t>
+        </is>
+      </c>
+      <c r="I74" s="20" t="inlineStr">
+        <is>
+          <t>亮铂金、典雅黑</t>
+        </is>
+      </c>
+      <c r="J74" s="20" t="inlineStr">
+        <is>
+          <t>12.3 英寸 PixelSense™ 显示屏 | 2736 × 1824 | 60Hz (防反射高透 LCD)</t>
+        </is>
+      </c>
+      <c r="K74" s="20" t="inlineStr">
+        <is>
+          <t>英特尔® 酷睿™ 第 8 代 i5-8350U (vPro) / i7-8650U (vPro)</t>
+        </is>
+      </c>
+      <c r="L74" s="20" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="M74" s="20" t="inlineStr">
+        <is>
+          <t>8GB / 16GB LPDDR3 | 128GB / 256GB / 512GB / 1TB PCIe NVMe SSD</t>
+        </is>
+      </c>
+      <c r="N74" s="20" t="inlineStr">
+        <is>
+          <t>常规使用约 13.5 小时</t>
+        </is>
+      </c>
+      <c r="O74" s="20" t="inlineStr">
+        <is>
+          <t>770g (i5) / 784g (i7)</t>
+        </is>
+      </c>
+      <c r="P74" s="20" t="inlineStr">
+        <is>
+          <t>Surface Pro 专业键盘盖 | 笔协议: 10 点触控，支持 Surface 触控笔 (4096 级压感)</t>
+        </is>
+      </c>
+      <c r="Q74" s="20" t="inlineStr">
+        <is>
+          <t>1 × 全尺寸 USB-A 3.0 + 1 × Mini DisplayPort + 1 × Surface Connect; 雷电: not_applicable; 磁吸: 配备经典磁吸 Surface Connect 口</t>
+        </is>
+      </c>
+      <c r="R74" s="23" t="inlineStr">
+        <is>
+          <t>点击进入商城选配 ↗</t>
+        </is>
+      </c>
+      <c r="S74" s="23" t="inlineStr">
+        <is>
+          <t>点击查阅架构白皮书 ↗</t>
+        </is>
+      </c>
+      <c r="T74" s="20" t="inlineStr">
+        <is>
+          <t>microsoft_official</t>
+        </is>
+      </c>
+      <c r="U74" s="21" t="inlineStr">
         <is>
           <t>✅ 100% 官方已核验</t>
         </is>
@@ -7593,6 +8223,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S67" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R68" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S68" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R69" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S69" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R70" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S70" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R71" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S71" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R72" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S72" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R73" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S73" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R74" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S74" r:id="rId140"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7711,7 +8353,7 @@
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>¥16,888 起 (商用)</t>
+          <t>¥13,588 起 (商用版)</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
@@ -7773,7 +8415,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>¥15,488 起 (商用)</t>
+          <t>¥13,588 起 (商用版)</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
@@ -7897,7 +8539,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>9,888 起 (商用)</t>
+          <t>¥12,288 起 (商用版)</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -7959,7 +8601,7 @@
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>¥16,888 起 (商用)</t>
+          <t>¥15,388 起 (商用版)</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -8021,7 +8663,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>¥14,888 起 (商用)</t>
+          <t>¥13,188 起 (商用版)</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -8083,7 +8725,7 @@
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>¥18,888 起 (商用)</t>
+          <t>¥17,588 起 (商用版)</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
@@ -8145,7 +8787,7 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>¥16,888 起 (商用)</t>
+          <t>¥16,488 起 (商用版)</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -8207,7 +8849,7 @@
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>9,988 起</t>
+          <t>¥12,288 起 (商用版)</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">

</xml_diff>